<commit_message>
chore: daily SAM report 2026-07-16
</commit_message>
<xml_diff>
--- a/docs/v/SAM-daily-latest.xlsx
+++ b/docs/v/SAM-daily-latest.xlsx
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>50</v>
@@ -12048,7 +12048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -12118,7 +12118,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>2026-07-16_102825</t>
+          <t>2026-07-16_110257</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
@@ -12156,7 +12156,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>2026-07-16_020140</t>
+          <t>2026-07-16_102825</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -12181,7 +12181,7 @@
         <v>50</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="H3" s="6" t="n">
         <v>3</v>
@@ -12194,7 +12194,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-16_015238</t>
+          <t>2026-07-16_020140</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -12204,7 +12204,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -12216,10 +12216,10 @@
         <v>22</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>1</v>
+        <v>49</v>
       </c>
       <c r="H4" s="6" t="n">
         <v>3</v>
@@ -12227,7 +12227,45 @@
       <c r="I4" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16_015238</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>API term='ArcPoint': HTTP 429 for https://api.sam.gov/prod/opportunities/v2/search?api_key=***: {"code":"900804","message":"Message throttled out","description":"You have exceeded your quota .You can access API after 2026-Jul-17 00:00:00+0000 UTC","nextAccessTime":"2026-Jul-17 00:00:00+0000 UTC"}</t>
         </is>

</xml_diff>